<commit_message>
Updated SNF, NEMO, ANF and ab-SNF silhouettes; done
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/NEMO/NEMO_TCGA_RNAseq-CNV-Methylation-miRNA-SNPs_eval_on_transNEO_clusterings.xlsx
+++ b/Results/single_algorithm/NEMO/NEMO_TCGA_RNAseq-CNV-Methylation-miRNA-SNPs_eval_on_transNEO_clusterings.xlsx
@@ -2384,7 +2384,7 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -2456,7 +2456,7 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -2672,7 +2672,7 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57">
@@ -3064,7 +3064,7 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="106">
@@ -3224,7 +3224,7 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126">
@@ -3488,7 +3488,7 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="159">
@@ -4584,7 +4584,7 @@
         <v>297</v>
       </c>
       <c r="B295" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="296">
@@ -4784,7 +4784,7 @@
         <v>322</v>
       </c>
       <c r="B320" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="321">
@@ -5120,7 +5120,7 @@
         <v>364</v>
       </c>
       <c r="B362" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="363">
@@ -5784,7 +5784,7 @@
         <v>447</v>
       </c>
       <c r="B445" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="446">
@@ -5864,7 +5864,7 @@
         <v>457</v>
       </c>
       <c r="B455" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="456">
@@ -5880,7 +5880,7 @@
         <v>459</v>
       </c>
       <c r="B457" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="458">
@@ -6624,7 +6624,7 @@
         <v>552</v>
       </c>
       <c r="B550" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="551">
@@ -6776,7 +6776,7 @@
         <v>571</v>
       </c>
       <c r="B569" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="570">
@@ -6904,7 +6904,7 @@
         <v>587</v>
       </c>
       <c r="B585" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="586">

</xml_diff>